<commit_message>
Compare the field list to the n8n QBO Estimate Intake data table
New Intake Table Gap tab maps all 46 data points and all 29 intake
columns: matches, gaps, items the flow can set itself, and columns that
aren't on the list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsQri8ybXXT892hQrSQMgg
</commit_message>
<xml_diff>
--- a/docs/qbo_customer_project_estimate_fields.xlsx
+++ b/docs/qbo_customer_project_estimate_fields.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Field List" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Estimate Comparison" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Excluded" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Intake Table Gap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Excluded" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Field List'!$A$4:$S$65</definedName>
@@ -88,7 +89,7 @@
       <color rgb="001F4E78"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -155,6 +156,21 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -182,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -264,7 +280,25 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5995,6 +6029,1293 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>QBO Estimate Intake (n8n data table) vs. the field list</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Compares data table Z3FW8RjSWUyDcIBl (29 columns, 0 rows as of 2026-09-24) to the 46 data points on the Field List tab. Status counts are formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Field List data point</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Intake table column</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Your decision</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>Customer (parent) name</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>customer_name</t>
+        </is>
+      </c>
+      <c r="C5" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="37" t="n"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Match (incl. output)</t>
+        </is>
+      </c>
+      <c r="H5" s="4">
+        <f>COUNTIF($C$5:$C$62,"Match*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Company name</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>customer_company</t>
+        </is>
+      </c>
+      <c r="C6" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="37" t="n"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H6" s="4">
+        <f>COUNTIF($C$5:$C$62,"Partial")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Customer group (parent's parent)</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="n"/>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Only needed when the parent is under a larger company (1/5).</t>
+        </is>
+      </c>
+      <c r="E7" s="37" t="n"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="H7" s="4">
+        <f>COUNTIF($C$5:$C$62,"Missing")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Contact first / last name</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="n"/>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>Optional (1/5).</t>
+        </is>
+      </c>
+      <c r="E8" s="37" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="H8" s="4">
+        <f>COUNTIF($C$5:$C$62,"Set by flow")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Customer email(s)</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>customer_email</t>
+        </is>
+      </c>
+      <c r="C9" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>Allow several addresses separated by commas.</t>
+        </is>
+      </c>
+      <c r="E9" s="37" t="n"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="H9" s="4">
+        <f>COUNTIF($C$5:$C$62,"In table, not on list")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Customer phone</t>
+        </is>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>customer_phone</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="37" t="n"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Tracking column</t>
+        </is>
+      </c>
+      <c r="H10" s="4">
+        <f>COUNTIF($C$5:$C$62,"Tracking column")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>Billing street</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="n"/>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5. Needed to create a new customer and for the estimate bill-to.</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>Billing city</t>
+        </is>
+      </c>
+      <c r="B12" s="32" t="n"/>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5.</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>Billing state</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="n"/>
+      <c r="C13" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5.</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>Billing ZIP</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="n"/>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5.</t>
+        </is>
+      </c>
+      <c r="E14" s="37" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>Ship-to name</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="n"/>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>Used 4/5. Company name or 'Local Pickup'.</t>
+        </is>
+      </c>
+      <c r="E15" s="37" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>Ship-to street</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="n"/>
+      <c r="C16" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5. Job site, the dealer's address, or Local Pickup.</t>
+        </is>
+      </c>
+      <c r="E16" s="37" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>Ship-to city, state, ZIP</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="n"/>
+      <c r="C17" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5.</t>
+        </is>
+      </c>
+      <c r="E17" s="37" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>Sales tax exempt?</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="n"/>
+      <c r="C18" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5. Decides whether a Sales Tax fee line is added. (tax_code looks like the per-line TAX/NON code.)</t>
+        </is>
+      </c>
+      <c r="E18" s="37" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>Resale / exemption number</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>Used 2/5, on exempt customers.</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>Customer notes</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>Optional (3/5).</t>
+        </is>
+      </c>
+      <c r="E20" s="37" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>Customer type</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>Optional (1/5).</t>
+        </is>
+      </c>
+      <c r="E21" s="37" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>Tax code</t>
+        </is>
+      </c>
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>Always 999. Doesn't need a column.</t>
+        </is>
+      </c>
+      <c r="E22" s="37" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="35" t="inlineStr">
+        <is>
+          <t>Payment terms</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="n"/>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>Company default, per your instruction.</t>
+        </is>
+      </c>
+      <c r="E23" s="37" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>Preferred delivery method</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="n"/>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>Always Print.</t>
+        </is>
+      </c>
+      <c r="E24" s="37" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="35" t="inlineStr">
+        <is>
+          <t>Customer message</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D25" s="32" t="inlineStr">
+        <is>
+          <t>QBO fills in the default.</t>
+        </is>
+      </c>
+      <c r="E25" s="37" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>Accounting email (Bcc)</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="inlineStr">
+        <is>
+          <t>Always Accounting@panda-windows.com.</t>
+        </is>
+      </c>
+      <c r="E26" s="37" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="35" t="inlineStr">
+        <is>
+          <t>Project / job name</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>project_name</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="37" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>Sub-customer flag</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="n"/>
+      <c r="C28" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>Always true.</t>
+        </is>
+      </c>
+      <c r="E28" s="37" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>Bill with parent</t>
+        </is>
+      </c>
+      <c r="B29" s="32" t="n"/>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D29" s="32" t="inlineStr">
+        <is>
+          <t>Always true.</t>
+        </is>
+      </c>
+      <c r="E29" s="37" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="35" t="inlineStr">
+        <is>
+          <t>QBO Project link</t>
+        </is>
+      </c>
+      <c r="B30" s="32" t="inlineStr">
+        <is>
+          <t>project_ref_id / native_project_id</t>
+        </is>
+      </c>
+      <c r="C30" s="36" t="inlineStr">
+        <is>
+          <t>Match (output)</t>
+        </is>
+      </c>
+      <c r="D30" s="32" t="inlineStr">
+        <is>
+          <t>The flow writes these back. The true Project still has to be created in QBO first.</t>
+        </is>
+      </c>
+      <c r="E30" s="37" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="35" t="inlineStr">
+        <is>
+          <t>Estimate #</t>
+        </is>
+      </c>
+      <c r="B31" s="32" t="inlineStr">
+        <is>
+          <t>doc_number (input) / estimate_doc_number (output)</t>
+        </is>
+      </c>
+      <c r="C31" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="37" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="35" t="inlineStr">
+        <is>
+          <t>Estimate date</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="n"/>
+      <c r="C32" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D32" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5. The flow could default to today, but the dates on the samples were all different.</t>
+        </is>
+      </c>
+      <c r="E32" s="37" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="35" t="inlineStr">
+        <is>
+          <t>Sales rep email(s) (Cc)</t>
+        </is>
+      </c>
+      <c r="B33" s="32" t="n"/>
+      <c r="C33" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D33" s="32" t="inlineStr">
+        <is>
+          <t>Used 5/5, and it's how reps are tied to estimates. rsm and outside_sales_rep hold names, not the Cc email.</t>
+        </is>
+      </c>
+      <c r="E33" s="37" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="35" t="inlineStr">
+        <is>
+          <t>Q Number / PO #</t>
+        </is>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>q_number_po</t>
+        </is>
+      </c>
+      <c r="C34" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D34" s="32" t="n"/>
+      <c r="E34" s="37" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>Deposit Due</t>
+        </is>
+      </c>
+      <c r="B35" s="32" t="inlineStr">
+        <is>
+          <t>deposit_due</t>
+        </is>
+      </c>
+      <c r="C35" s="36" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D35" s="32" t="inlineStr">
+        <is>
+          <t>Free text.</t>
+        </is>
+      </c>
+      <c r="E35" s="37" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>Product / Service</t>
+        </is>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>item_ref_id + line_items_json</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D36" s="32" t="inlineStr">
+        <is>
+          <t>The item_* columns hold only ONE line. The samples had 3–13 lines, so line_items_json has to carry them.</t>
+        </is>
+      </c>
+      <c r="E36" s="37" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>Line description</t>
+        </is>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>item_description + line_items_json</t>
+        </is>
+      </c>
+      <c r="C37" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D37" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E37" s="37" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="35" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B38" s="32" t="inlineStr">
+        <is>
+          <t>item_qty + line_items_json</t>
+        </is>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D38" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E38" s="37" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>item_unit_price + line_items_json</t>
+        </is>
+      </c>
+      <c r="C39" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D39" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E39" s="37" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="35" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="B40" s="32" t="inlineStr">
+        <is>
+          <t>item_amount + line_items_json</t>
+        </is>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D40" s="32" t="inlineStr">
+        <is>
+          <t>Could be calculated as qty × rate.</t>
+        </is>
+      </c>
+      <c r="E40" s="37" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="35" t="inlineStr">
+        <is>
+          <t>Line tax code</t>
+        </is>
+      </c>
+      <c r="B41" s="32" t="inlineStr">
+        <is>
+          <t>tax_code + line_items_json</t>
+        </is>
+      </c>
+      <c r="C41" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D41" s="32" t="inlineStr">
+        <is>
+          <t>Needs a value per line (TAX vs NON).</t>
+        </is>
+      </c>
+      <c r="E41" s="37" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="35" t="inlineStr">
+        <is>
+          <t>Line dimension 1000000039</t>
+        </is>
+      </c>
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>(line_items_json?)</t>
+        </is>
+      </c>
+      <c r="C42" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D42" s="32" t="inlineStr">
+        <is>
+          <t>On every product line. No column, and the JSON layout isn't defined.</t>
+        </is>
+      </c>
+      <c r="E42" s="37" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>Line dimension 1000000051</t>
+        </is>
+      </c>
+      <c r="B43" s="32" t="inlineStr">
+        <is>
+          <t>(line_items_json?)</t>
+        </is>
+      </c>
+      <c r="C43" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D43" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E43" s="37" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="35" t="inlineStr">
+        <is>
+          <t>Line dimension 1000000172</t>
+        </is>
+      </c>
+      <c r="B44" s="32" t="inlineStr">
+        <is>
+          <t>(line_items_json?)</t>
+        </is>
+      </c>
+      <c r="C44" s="38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D44" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E44" s="37" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="35" t="inlineStr">
+        <is>
+          <t>Crating fee</t>
+        </is>
+      </c>
+      <c r="B45" s="32" t="inlineStr">
+        <is>
+          <t>(line_items_json?)</t>
+        </is>
+      </c>
+      <c r="C45" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D45" s="32" t="inlineStr">
+        <is>
+          <t>Can go in line_items_json as a 'Z Fees:Crating' line, or get its own column. Used 4/5.</t>
+        </is>
+      </c>
+      <c r="E45" s="37" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>Shipping fee</t>
+        </is>
+      </c>
+      <c r="B46" s="32" t="inlineStr">
+        <is>
+          <t>(line_items_json?)</t>
+        </is>
+      </c>
+      <c r="C46" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D46" s="32" t="inlineStr">
+        <is>
+          <t>Same, 'Z Fees:Shipping Fee' (NON). Used 4/5.</t>
+        </is>
+      </c>
+      <c r="E46" s="37" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="35" t="inlineStr">
+        <is>
+          <t>Sales tax line</t>
+        </is>
+      </c>
+      <c r="B47" s="32" t="inlineStr">
+        <is>
+          <t>(line_items_json?)</t>
+        </is>
+      </c>
+      <c r="C47" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D47" s="32" t="inlineStr">
+        <is>
+          <t>Same, 'Z Fees:Sales Tax' (NON). Used 2/5.</t>
+        </is>
+      </c>
+      <c r="E47" s="37" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>Soft wrap fee</t>
+        </is>
+      </c>
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>(line_items_json?)</t>
+        </is>
+      </c>
+      <c r="C48" s="40" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D48" s="32" t="inlineStr">
+        <is>
+          <t>Same, 'Z Fees:Soft Wrap'. Used 1/5.</t>
+        </is>
+      </c>
+      <c r="E48" s="37" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="35" t="inlineStr">
+        <is>
+          <t>Deposit placeholder line</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="n"/>
+      <c r="C49" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D49" s="32" t="inlineStr">
+        <is>
+          <t>$0 'Z Fees:Deposit' line.</t>
+        </is>
+      </c>
+      <c r="E49" s="37" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>Subtotal line</t>
+        </is>
+      </c>
+      <c r="B50" s="32" t="n"/>
+      <c r="C50" s="39" t="inlineStr">
+        <is>
+          <t>Set by flow</t>
+        </is>
+      </c>
+      <c r="D50" s="32" t="n"/>
+      <c r="E50" s="37" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>Columns in the intake table that aren't on the field list</t>
+        </is>
+      </c>
+      <c r="B51" s="30" t="n"/>
+      <c r="C51" s="30" t="n"/>
+      <c r="D51" s="30" t="n"/>
+      <c r="E51" s="30" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="32" t="n"/>
+      <c r="B52" s="35" t="inlineStr">
+        <is>
+          <t>project_start_date</t>
+        </is>
+      </c>
+      <c r="C52" s="41" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="D52" s="32" t="inlineStr">
+        <is>
+          <t>QBO's REST API can't set project dates, and none of the samples had them. Drop the column, or write the dates by hand in QBO.</t>
+        </is>
+      </c>
+      <c r="E52" s="37" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="32" t="n"/>
+      <c r="B53" s="35" t="inlineStr">
+        <is>
+          <t>project_end_date</t>
+        </is>
+      </c>
+      <c r="C53" s="41" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="D53" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E53" s="37" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="32" t="n"/>
+      <c r="B54" s="35" t="inlineStr">
+        <is>
+          <t>estimate_memo</t>
+        </is>
+      </c>
+      <c r="C54" s="41" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="D54" s="32" t="inlineStr">
+        <is>
+          <t>None of the 5 had an internal memo, and the customer message is always the default. Keep it only if you plan to use it.</t>
+        </is>
+      </c>
+      <c r="E54" s="37" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="32" t="n"/>
+      <c r="B55" s="35" t="inlineStr">
+        <is>
+          <t>residential_or_commercial</t>
+        </is>
+      </c>
+      <c r="C55" s="41" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="D55" s="32" t="inlineStr">
+        <is>
+          <t>Newer custom field. Writing it through the v3 API didn't save (tests 66–76), and it's blank on every row of the QBO Estimates table. It needs GraphQL access.</t>
+        </is>
+      </c>
+      <c r="E55" s="37" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="32" t="n"/>
+      <c r="B56" s="35" t="inlineStr">
+        <is>
+          <t>dealer</t>
+        </is>
+      </c>
+      <c r="C56" s="41" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="D56" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E56" s="37" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="32" t="n"/>
+      <c r="B57" s="35" t="inlineStr">
+        <is>
+          <t>rsm</t>
+        </is>
+      </c>
+      <c r="C57" s="41" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="D57" s="32" t="inlineStr">
+        <is>
+          <t>Same as above.</t>
+        </is>
+      </c>
+      <c r="E57" s="37" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="32" t="n"/>
+      <c r="B58" s="35" t="inlineStr">
+        <is>
+          <t>outside_sales_rep</t>
+        </is>
+      </c>
+      <c r="C58" s="41" t="inlineStr">
+        <is>
+          <t>In table, not on list</t>
+        </is>
+      </c>
+      <c r="D58" s="32" t="inlineStr">
+        <is>
+          <t>Same as above. The samples track reps with the Cc email instead.</t>
+        </is>
+      </c>
+      <c r="E58" s="37" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="32" t="n"/>
+      <c r="B59" s="35" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C59" s="39" t="inlineStr">
+        <is>
+          <t>Tracking column</t>
+        </is>
+      </c>
+      <c r="D59" s="32" t="inlineStr">
+        <is>
+          <t>Workflow status, e.g. pending / done / error.</t>
+        </is>
+      </c>
+      <c r="E59" s="37" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="32" t="n"/>
+      <c r="B60" s="35" t="inlineStr">
+        <is>
+          <t>customer_ref_id</t>
+        </is>
+      </c>
+      <c r="C60" s="39" t="inlineStr">
+        <is>
+          <t>Tracking column</t>
+        </is>
+      </c>
+      <c r="D60" s="32" t="inlineStr">
+        <is>
+          <t>The flow writes back the QBO customer Id.</t>
+        </is>
+      </c>
+      <c r="E60" s="37" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="32" t="n"/>
+      <c r="B61" s="35" t="inlineStr">
+        <is>
+          <t>estimate_id</t>
+        </is>
+      </c>
+      <c r="C61" s="39" t="inlineStr">
+        <is>
+          <t>Tracking column</t>
+        </is>
+      </c>
+      <c r="D61" s="32" t="inlineStr">
+        <is>
+          <t>The flow writes back the QBO estimate Id.</t>
+        </is>
+      </c>
+      <c r="E61" s="37" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="32" t="n"/>
+      <c r="B62" s="35" t="inlineStr">
+        <is>
+          <t>last_error</t>
+        </is>
+      </c>
+      <c r="C62" s="39" t="inlineStr">
+        <is>
+          <t>Tracking column</t>
+        </is>
+      </c>
+      <c r="D62" s="32" t="inlineStr">
+        <is>
+          <t>The flow's error message.</t>
+        </is>
+      </c>
+      <c r="E62" s="37" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E5:E62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Add column,Put in line_items_json,Set in flow,Drop column,Keep as is"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6056,7 +7377,7 @@
           <t>0/5</t>
         </is>
       </c>
-      <c r="D5" s="35" t="n"/>
+      <c r="D5" s="37" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="32" t="inlineStr">
@@ -6074,7 +7395,7 @@
           <t>0/5</t>
         </is>
       </c>
-      <c r="D6" s="35" t="n"/>
+      <c r="D6" s="37" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="32" t="inlineStr">
@@ -6092,7 +7413,7 @@
           <t>0/5 (and dates can't be set through the API)</t>
         </is>
       </c>
-      <c r="D7" s="35" t="n"/>
+      <c r="D7" s="37" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="32" t="inlineStr">
@@ -6110,7 +7431,7 @@
           <t>0/5</t>
         </is>
       </c>
-      <c r="D8" s="35" t="n"/>
+      <c r="D8" s="37" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="32" t="inlineStr">
@@ -6128,7 +7449,7 @@
           <t>0/5</t>
         </is>
       </c>
-      <c r="D9" s="35" t="n"/>
+      <c r="D9" s="37" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="32" t="inlineStr">
@@ -6146,7 +7467,7 @@
           <t>0/5</t>
         </is>
       </c>
-      <c r="D10" s="35" t="n"/>
+      <c r="D10" s="37" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="32" t="inlineStr">
@@ -6164,7 +7485,7 @@
           <t>0/5</t>
         </is>
       </c>
-      <c r="D11" s="35" t="n"/>
+      <c r="D11" s="37" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="32" t="inlineStr">
@@ -6182,7 +7503,7 @@
           <t>0/5 (1 of the earlier 10 had one)</t>
         </is>
       </c>
-      <c r="D12" s="35" t="n"/>
+      <c r="D12" s="37" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="32" t="inlineStr">
@@ -6200,7 +7521,7 @@
           <t>0/5. Shipping and deposit are handled as fee lines and the Deposit Due field.</t>
         </is>
       </c>
-      <c r="D13" s="35" t="n"/>
+      <c r="D13" s="37" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="32" t="inlineStr">
@@ -6218,7 +7539,7 @@
           <t>0/5. Reps are tracked with the Cc email.</t>
         </is>
       </c>
-      <c r="D14" s="35" t="n"/>
+      <c r="D14" s="37" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="32" t="inlineStr">
@@ -6236,7 +7557,7 @@
           <t>Can't be read or written through our current API. If your team fills these in on screen, move them back to the main list.</t>
         </is>
       </c>
-      <c r="D15" s="35" t="n"/>
+      <c r="D15" s="37" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="32" t="inlineStr">
@@ -6254,7 +7575,7 @@
           <t>QBO sets these after the estimate is created (4/5 were converted to invoices).</t>
         </is>
       </c>
-      <c r="D16" s="35" t="n"/>
+      <c r="D16" s="37" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>